<commit_message>
Limpia .gitignore y elimina archivos de Visual Studio
</commit_message>
<xml_diff>
--- a/backend/app/REGISTRO ACADEMICO ROSTER.xlsx
+++ b/backend/app/REGISTRO ACADEMICO ROSTER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\proyecto\Registro_academico\backend\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CA008C6-4D19-46FD-9431-8F39763A362A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8DB8ACD-4EDC-46E9-A960-0D3AED35664A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="18000" windowHeight="9270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ROSTER REGISTRO ACADEMICO" sheetId="1" r:id="rId1"/>
@@ -2862,13 +2862,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:XFD503"/>
+  <dimension ref="A1:XFC503"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
     <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="8.28515625" customWidth="1"/>
     <col min="6" max="6" width="16.85546875" customWidth="1"/>
     <col min="7" max="7" width="11.42578125" style="9" customWidth="1"/>
@@ -5133,7 +5133,7 @@
         <v>6</v>
       </c>
       <c r="E120" s="13" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F120" s="13"/>
       <c r="G120" s="18">

</xml_diff>